<commit_message>
fix bug completion rate
</commit_message>
<xml_diff>
--- a/src/main/kotlin/com/kcvn/spm/assets/template/ExportCompletionProcessProductRateTemplate.xlsx
+++ b/src/main/kotlin/com/kcvn/spm/assets/template/ExportCompletionProcessProductRateTemplate.xlsx
@@ -47,7 +47,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -71,10 +71,18 @@
       <family val="0"/>
     </font>
     <font>
-      <sz val="11"/>
+      <sz val="12"/>
       <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="0"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -120,12 +128,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -147,32 +159,33 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F1"/>
-  <sheetFormatPr defaultColWidth="12.640625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.66015625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="21.81"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="23.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="28.2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14.59"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26.39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="20.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="23.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="28.19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="14.59"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="12.64"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>